<commit_message>
chore: sync Nova upm-release-2026.08.14-03
</commit_message>
<xml_diff>
--- a/Assets/Samples/IAPDemo/Excels/Networks/HostKeys/NetworkHostKeys.xlsx
+++ b/Assets/Samples/IAPDemo/Excels/Networks/HostKeys/NetworkHostKeys.xlsx
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="58" uniqueCount="26">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="74" uniqueCount="29">
   <si>
     <t>##comment</t>
   </si>
@@ -106,6 +106,15 @@
   <si>
     <t>https://t-payments.solotopiax.com</t>
     <phoneticPr fontId="4" type="noConversion"/>
+  </si>
+  <si>
+    <t>FallbackValue</t>
+  </si>
+  <si>
+    <t>主域名</t>
+  </si>
+  <si>
+    <t>备用域名</t>
   </si>
 </sst>
 </file>
@@ -620,7 +629,9 @@
       <c r="D2" s="5" t="s">
         <v>5</v>
       </c>
-      <c r="E2" s="5"/>
+      <c r="E2" s="5" t="s">
+        <v>26</v>
+      </c>
       <c r="F2" s="5"/>
       <c r="G2" s="5"/>
       <c r="H2" s="5"/>
@@ -654,7 +665,9 @@
       <c r="D3" s="6" t="s">
         <v>7</v>
       </c>
-      <c r="E3" s="6"/>
+      <c r="E3" s="6" t="s">
+        <v>7</v>
+      </c>
       <c r="F3" s="6"/>
       <c r="G3" s="6"/>
       <c r="H3" s="6"/>
@@ -686,7 +699,10 @@
         <v>9</v>
       </c>
       <c r="D4" s="1" t="s">
-        <v>10</v>
+        <v>27</v>
+      </c>
+      <c r="E4" s="1" t="s">
+        <v>28</v>
       </c>
     </row>
     <row r="5" spans="1:24" ht="22" customHeight="1" x14ac:dyDescent="0.25">
@@ -699,6 +715,9 @@
       <c r="D5" s="7" t="s">
         <v>13</v>
       </c>
+      <c r="E5" s="7" t="s">
+        <v>13</v>
+      </c>
     </row>
     <row r="6" spans="1:24" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B6" s="3" t="s">
@@ -710,6 +729,9 @@
       <c r="D6" s="7" t="s">
         <v>15</v>
       </c>
+      <c r="E6" s="7" t="s">
+        <v>15</v>
+      </c>
     </row>
     <row r="7" spans="1:24" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B7" s="8" t="s">
@@ -721,6 +743,9 @@
       <c r="D7" s="7" t="s">
         <v>22</v>
       </c>
+      <c r="E7" s="7" t="s">
+        <v>22</v>
+      </c>
     </row>
     <row r="8" spans="1:24" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B8" s="8" t="s">
@@ -732,6 +757,9 @@
       <c r="D8" s="7" t="s">
         <v>22</v>
       </c>
+      <c r="E8" s="7" t="s">
+        <v>22</v>
+      </c>
     </row>
     <row r="9" spans="1:24" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B9" s="8" t="s">
@@ -741,6 +769,9 @@
         <v>24</v>
       </c>
       <c r="D9" s="7" t="s">
+        <v>25</v>
+      </c>
+      <c r="E9" s="7" t="s">
         <v>25</v>
       </c>
     </row>
@@ -782,10 +813,15 @@
   <phoneticPr fontId="4" type="noConversion"/>
   <hyperlinks>
     <hyperlink ref="D5" r:id="rId1" tooltip="https://t-solo-api-game.ahameet.com" xr:uid="{00000000-0004-0000-0000-000000000000}"/>
+    <hyperlink ref="E5" r:id="rId1" tooltip="https://t-solo-api-game.ahameet.com" xr:uid="{00000000-0004-0000-0000-000000000000}"/>
     <hyperlink ref="D6" r:id="rId2" xr:uid="{00000000-0004-0000-0000-000001000000}"/>
+    <hyperlink ref="E6" r:id="rId2" xr:uid="{00000000-0004-0000-0000-000001000000}"/>
     <hyperlink ref="D7" r:id="rId3" xr:uid="{00000000-0004-0000-0000-000002000000}"/>
+    <hyperlink ref="E7" r:id="rId3" xr:uid="{00000000-0004-0000-0000-000002000000}"/>
     <hyperlink ref="D8" r:id="rId4" xr:uid="{4A9895B5-FA1E-4E9B-8ADC-D73489DFF848}"/>
+    <hyperlink ref="E8" r:id="rId4" xr:uid="{4A9895B5-FA1E-4E9B-8ADC-D73489DFF848}"/>
     <hyperlink ref="D9" r:id="rId5" xr:uid="{06AC7C6F-AF32-4044-A73C-25DBBC2FF81A}"/>
+    <hyperlink ref="E9" r:id="rId5" xr:uid="{06AC7C6F-AF32-4044-A73C-25DBBC2FF81A}"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId6"/>
@@ -846,7 +882,9 @@
       <c r="D2" s="5" t="s">
         <v>5</v>
       </c>
-      <c r="E2" s="5"/>
+      <c r="E2" s="5" t="s">
+        <v>26</v>
+      </c>
       <c r="F2" s="5"/>
       <c r="G2" s="5"/>
       <c r="H2" s="5"/>
@@ -880,7 +918,9 @@
       <c r="D3" s="6" t="s">
         <v>7</v>
       </c>
-      <c r="E3" s="6"/>
+      <c r="E3" s="6" t="s">
+        <v>7</v>
+      </c>
       <c r="F3" s="6"/>
       <c r="G3" s="6"/>
       <c r="H3" s="6"/>
@@ -912,7 +952,10 @@
         <v>9</v>
       </c>
       <c r="D4" s="1" t="s">
-        <v>10</v>
+        <v>27</v>
+      </c>
+      <c r="E4" s="1" t="s">
+        <v>28</v>
       </c>
     </row>
     <row r="5" spans="1:24" ht="22" customHeight="1" x14ac:dyDescent="0.25">
@@ -925,6 +968,9 @@
       <c r="D5" s="7" t="s">
         <v>13</v>
       </c>
+      <c r="E5" s="7" t="s">
+        <v>13</v>
+      </c>
     </row>
     <row r="6" spans="1:24" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B6" s="3" t="s">
@@ -936,6 +982,9 @@
       <c r="D6" s="7" t="s">
         <v>15</v>
       </c>
+      <c r="E6" s="7" t="s">
+        <v>15</v>
+      </c>
     </row>
     <row r="7" spans="1:24" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B7" s="8" t="s">
@@ -947,6 +996,9 @@
       <c r="D7" s="7" t="s">
         <v>18</v>
       </c>
+      <c r="E7" s="7" t="s">
+        <v>18</v>
+      </c>
     </row>
     <row r="8" spans="1:24" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B8" s="8" t="s">
@@ -958,6 +1010,9 @@
       <c r="D8" s="7" t="s">
         <v>22</v>
       </c>
+      <c r="E8" s="7" t="s">
+        <v>22</v>
+      </c>
     </row>
     <row r="9" spans="1:24" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B9" s="8" t="s">
@@ -967,6 +1022,9 @@
         <v>24</v>
       </c>
       <c r="D9" s="7" t="s">
+        <v>25</v>
+      </c>
+      <c r="E9" s="7" t="s">
         <v>25</v>
       </c>
     </row>
@@ -1008,10 +1066,15 @@
   <phoneticPr fontId="4" type="noConversion"/>
   <hyperlinks>
     <hyperlink ref="D5" r:id="rId1" tooltip="https://t-solo-api-game.ahameet.com" xr:uid="{00000000-0004-0000-0100-000000000000}"/>
+    <hyperlink ref="E5" r:id="rId1" tooltip="https://t-solo-api-game.ahameet.com" xr:uid="{00000000-0004-0000-0100-000000000000}"/>
     <hyperlink ref="D6" r:id="rId2" xr:uid="{00000000-0004-0000-0100-000001000000}"/>
+    <hyperlink ref="E6" r:id="rId2" xr:uid="{00000000-0004-0000-0100-000001000000}"/>
     <hyperlink ref="D7" r:id="rId3" xr:uid="{00000000-0004-0000-0100-000002000000}"/>
+    <hyperlink ref="E7" r:id="rId3" xr:uid="{00000000-0004-0000-0100-000002000000}"/>
     <hyperlink ref="D8" r:id="rId4" xr:uid="{1585AF03-04DA-47C6-A7C9-D24FB2F8CA60}"/>
+    <hyperlink ref="E8" r:id="rId4" xr:uid="{1585AF03-04DA-47C6-A7C9-D24FB2F8CA60}"/>
     <hyperlink ref="D9" r:id="rId5" xr:uid="{36AA8FA0-9428-43BB-99F6-0B30FB88A3CD}"/>
+    <hyperlink ref="E9" r:id="rId5" xr:uid="{36AA8FA0-9428-43BB-99F6-0B30FB88A3CD}"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup paperSize="9" orientation="portrait"/>

</xml_diff>